<commit_message>
Add the extraction-loss columns to the Fig. 2(b)/2(c) workbook
The redrawn panel (c) shades eta_sub - EQE, so the workbook now carries
that difference as a formula column for each reflector rather than
leaving the reader to subtract.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A1WQ3WGcJw8tT3QK2n57xo
</commit_message>
<xml_diff>
--- a/figures/fig2b_mock/fig2bc_rawdata.xlsx
+++ b/figures/fig2b_mock/fig2bc_rawdata.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:B35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -639,120 +639,132 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
+          <t>extraction loss</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>eta_sub - EQE: what reached the substrate and never escaped.  This is the shaded band of panel (c).  FORMULA</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
           <t>p (flat interface)</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>reference column only, not used by any formula: the escape probability of a flat substrate/air interface for angularly randomised light, mean Fresnel transmittance over the escape cone divided by n_sub^2 (Yablonovitch 1982, one-sided)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Sheets</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>fig2b_2c</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>the plotted curves, with eta_ext and EQE as formulas</t>
+          <t>Sheets</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>Al_modes</t>
+          <t>fig2b_2c</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>the full five-channel power budget for the Al reflector, as the model returns it</t>
+          <t>the plotted curves, with eta_ext and EQE as formulas</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
+          <t>Al_modes</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>the full five-channel power budget for the Al reflector, as the model returns it</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
           <t>Ag_modes</t>
         </is>
       </c>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>the same for the Ag reflector</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>Provenance</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Script</t>
-        </is>
-      </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>sim/design_rule4/dr4f.m (Octave), MODE=nsub, run with UNUM=3000 and TOPMAT=al / ag</t>
+          <t>Provenance</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>Source files</t>
+          <t>Script</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>nsub_al_konig.csv and nsub_ag_konig.csv (model output), fig2b_curves_konig.csv (the assembled curves).  The earlier n = 1.9 + 0.02i run is kept alongside as nsub_{al,ag}.csv / fig2b_curves.csv</t>
+          <t>sim/design_rule4/dr4f.m (Octave), MODE=nsub, run with UNUM=3000 and TOPMAT=al / ag</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>p</t>
+          <t>Source files</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>interpolated from the author's single-pass escape-probability curve: 0.665 / 0.470 / 0.380 / 0.355 / 0.335 / 0.305 / 0.275 / 0.248 at n_sub = 1.30 / 1.40 / 1.50 / 1.60 / 1.70 / 1.80 / 1.90 / 2.00</t>
+          <t>nsub_al_konig.csv and nsub_ag_konig.csv (model output), fig2b_curves_konig.csv (the assembled curves).  The earlier n = 1.9 + 0.02i run is kept alongside as nsub_{al,ag}.csv / fig2b_curves.csv</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Caution</t>
+          <t>p</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>column 9 of nsub_al_konig.csv and nsub_ag_konig.csv is eta_ext at the script's default p = 0.4 and is NOT the plotted curve; the workbook recomputes eta_ext from the p column</t>
+          <t>interpolated from the author's single-pass escape-probability curve: 0.665 / 0.470 / 0.380 / 0.355 / 0.335 / 0.305 / 0.275 / 0.248 at n_sub = 1.30 / 1.40 / 1.50 / 1.60 / 1.70 / 1.80 / 1.90 / 2.00</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
+          <t>Caution</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>column 9 of nsub_al_konig.csv and nsub_ag_konig.csv is eta_ext at the script's default p = 0.4 and is NOT the plotted curve; the workbook recomputes eta_ext from the p column</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
           <t>Repository</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>jjoono/OLED-, branch claude/oled-efficiency-paper-ag-955zsk, figures/fig2b_mock/</t>
         </is>
@@ -769,7 +781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -784,6 +796,8 @@
     <col width="14" customWidth="1" min="10" max="10"/>
     <col width="21" customWidth="1" min="11" max="11"/>
     <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="13" max="13"/>
+    <col width="21" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -796,7 +810,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>eta_ext = p/[p+(1-p)A'] and EQE = eta_sub x eta_ext are formulas; edit column B (yellow) to redraw with a different p</t>
+          <t>eta_ext, EQE and the two loss columns are formulas; edit column B (yellow) to redraw everything with a different p</t>
         </is>
       </c>
     </row>
@@ -857,6 +871,16 @@
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>extraction loss (Al)</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>extraction loss (Ag)</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>p, flat interface (reference)</t>
         </is>
@@ -901,7 +925,15 @@
         <f>I5-E5</f>
         <v/>
       </c>
-      <c r="L5" s="6" t="n">
+      <c r="L5" s="6">
+        <f>C5-F5</f>
+        <v/>
+      </c>
+      <c r="M5" s="6">
+        <f>G5-J5</f>
+        <v/>
+      </c>
+      <c r="N5" s="6" t="n">
         <v>0.5555426141807783</v>
       </c>
     </row>
@@ -944,7 +976,15 @@
         <f>I6-E6</f>
         <v/>
       </c>
-      <c r="L6" s="6" t="n">
+      <c r="L6" s="6">
+        <f>C6-F6</f>
+        <v/>
+      </c>
+      <c r="M6" s="6">
+        <f>G6-J6</f>
+        <v/>
+      </c>
+      <c r="N6" s="6" t="n">
         <v>0.5107915418560387</v>
       </c>
     </row>
@@ -987,7 +1027,15 @@
         <f>I7-E7</f>
         <v/>
       </c>
-      <c r="L7" s="6" t="n">
+      <c r="L7" s="6">
+        <f>C7-F7</f>
+        <v/>
+      </c>
+      <c r="M7" s="6">
+        <f>G7-J7</f>
+        <v/>
+      </c>
+      <c r="N7" s="6" t="n">
         <v>0.4710139087909155</v>
       </c>
     </row>
@@ -1030,7 +1078,15 @@
         <f>I8-E8</f>
         <v/>
       </c>
-      <c r="L8" s="6" t="n">
+      <c r="L8" s="6">
+        <f>C8-F8</f>
+        <v/>
+      </c>
+      <c r="M8" s="6">
+        <f>G8-J8</f>
+        <v/>
+      </c>
+      <c r="N8" s="6" t="n">
         <v>0.4354967086478286</v>
       </c>
     </row>
@@ -1073,7 +1129,15 @@
         <f>I9-E9</f>
         <v/>
       </c>
-      <c r="L9" s="6" t="n">
+      <c r="L9" s="6">
+        <f>C9-F9</f>
+        <v/>
+      </c>
+      <c r="M9" s="6">
+        <f>G9-J9</f>
+        <v/>
+      </c>
+      <c r="N9" s="6" t="n">
         <v>0.4036536942292964</v>
       </c>
     </row>
@@ -1116,7 +1180,15 @@
         <f>I10-E10</f>
         <v/>
       </c>
-      <c r="L10" s="6" t="n">
+      <c r="L10" s="6">
+        <f>C10-F10</f>
+        <v/>
+      </c>
+      <c r="M10" s="6">
+        <f>G10-J10</f>
+        <v/>
+      </c>
+      <c r="N10" s="6" t="n">
         <v>0.374998094679025</v>
       </c>
     </row>
@@ -1159,7 +1231,15 @@
         <f>I11-E11</f>
         <v/>
       </c>
-      <c r="L11" s="6" t="n">
+      <c r="L11" s="6">
+        <f>C11-F11</f>
+        <v/>
+      </c>
+      <c r="M11" s="6">
+        <f>G11-J11</f>
+        <v/>
+      </c>
+      <c r="N11" s="6" t="n">
         <v>0.3491223309818853</v>
       </c>
     </row>
@@ -1202,7 +1282,15 @@
         <f>I12-E12</f>
         <v/>
       </c>
-      <c r="L12" s="6" t="n">
+      <c r="L12" s="6">
+        <f>C12-F12</f>
+        <v/>
+      </c>
+      <c r="M12" s="6">
+        <f>G12-J12</f>
+        <v/>
+      </c>
+      <c r="N12" s="6" t="n">
         <v>0.3256826182327374</v>
       </c>
     </row>
@@ -1245,7 +1333,15 @@
         <f>I13-E13</f>
         <v/>
       </c>
-      <c r="L13" s="6" t="n">
+      <c r="L13" s="6">
+        <f>C13-F13</f>
+        <v/>
+      </c>
+      <c r="M13" s="6">
+        <f>G13-J13</f>
+        <v/>
+      </c>
+      <c r="N13" s="6" t="n">
         <v>0.3043870816108616</v>
       </c>
     </row>
@@ -1288,7 +1384,15 @@
         <f>I14-E14</f>
         <v/>
       </c>
-      <c r="L14" s="6" t="n">
+      <c r="L14" s="6">
+        <f>C14-F14</f>
+        <v/>
+      </c>
+      <c r="M14" s="6">
+        <f>G14-J14</f>
+        <v/>
+      </c>
+      <c r="N14" s="6" t="n">
         <v>0.284986457384909</v>
       </c>
     </row>
@@ -1331,7 +1435,15 @@
         <f>I15-E15</f>
         <v/>
       </c>
-      <c r="L15" s="6" t="n">
+      <c r="L15" s="6">
+        <f>C15-F15</f>
+        <v/>
+      </c>
+      <c r="M15" s="6">
+        <f>G15-J15</f>
+        <v/>
+      </c>
+      <c r="N15" s="6" t="n">
         <v>0.2672667313252264</v>
       </c>
     </row>
@@ -1374,7 +1486,15 @@
         <f>I16-E16</f>
         <v/>
       </c>
-      <c r="L16" s="6" t="n">
+      <c r="L16" s="6">
+        <f>C16-F16</f>
+        <v/>
+      </c>
+      <c r="M16" s="6">
+        <f>G16-J16</f>
+        <v/>
+      </c>
+      <c r="N16" s="6" t="n">
         <v>0.2510432517074033</v>
       </c>
     </row>
@@ -1417,7 +1537,15 @@
         <f>I17-E17</f>
         <v/>
       </c>
-      <c r="L17" s="6" t="n">
+      <c r="L17" s="6">
+        <f>C17-F17</f>
+        <v/>
+      </c>
+      <c r="M17" s="6">
+        <f>G17-J17</f>
+        <v/>
+      </c>
+      <c r="N17" s="6" t="n">
         <v>0.236155979456892</v>
       </c>
     </row>
@@ -1460,7 +1588,15 @@
         <f>I18-E18</f>
         <v/>
       </c>
-      <c r="L18" s="6" t="n">
+      <c r="L18" s="6">
+        <f>C18-F18</f>
+        <v/>
+      </c>
+      <c r="M18" s="6">
+        <f>G18-J18</f>
+        <v/>
+      </c>
+      <c r="N18" s="6" t="n">
         <v>0.2224656252191622</v>
       </c>
     </row>
@@ -1503,7 +1639,15 @@
         <f>I19-E19</f>
         <v/>
       </c>
-      <c r="L19" s="6" t="n">
+      <c r="L19" s="6">
+        <f>C19-F19</f>
+        <v/>
+      </c>
+      <c r="M19" s="6">
+        <f>G19-J19</f>
+        <v/>
+      </c>
+      <c r="N19" s="6" t="n">
         <v>0.2098504851395527</v>
       </c>
     </row>

</xml_diff>